<commit_message>
add simple new flowchart in xlsx
</commit_message>
<xml_diff>
--- a/Training_model/supplementary/Flowchart ML development.xlsx
+++ b/Training_model/supplementary/Flowchart ML development.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DeviceIdentifier\1.Training_model\supplementary\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DeviceIdentifier\Training_model\supplementary\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0212D06A-2953-471E-AFD8-776EEA1D0026}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CCFAA1C-CCE5-454E-AFA2-85B71C0368CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{A3A45E78-3C42-44AE-93A4-41B09245FE7F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{A3A45E78-3C42-44AE-93A4-41B09245FE7F}"/>
   </bookViews>
   <sheets>
     <sheet name="Flowchart ML" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="93">
   <si>
     <t>ALPHA_PREFIX_WEIGHT     = 0.65</t>
   </si>
@@ -314,7 +314,10 @@
     <t>ML pipeline workflow</t>
   </si>
   <si>
-    <t>Model Integration [28/08/2026]</t>
+    <t>Full Workflow Model Integration [28/08/2026]</t>
+  </si>
+  <si>
+    <t>Quick Overview</t>
   </si>
 </sst>
 </file>
@@ -361,7 +364,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -404,6 +407,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF002060"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -417,7 +426,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -448,10 +457,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -460,6 +469,10 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4154,7 +4167,7 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>47</xdr:col>
-      <xdr:colOff>61092</xdr:colOff>
+      <xdr:colOff>42042</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>85189</xdr:rowOff>
     </xdr:from>
@@ -4172,7 +4185,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="19452678" y="636982"/>
+          <a:off x="26896192" y="637639"/>
           <a:ext cx="1732998" cy="436786"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4258,7 +4271,7 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>47</xdr:col>
-      <xdr:colOff>398389</xdr:colOff>
+      <xdr:colOff>371174</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>87801</xdr:rowOff>
     </xdr:from>
@@ -4276,7 +4289,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="19789975" y="1375318"/>
+          <a:off x="27140960" y="1357801"/>
           <a:ext cx="1059934" cy="264560"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4332,7 +4345,7 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>47</xdr:col>
-      <xdr:colOff>53731</xdr:colOff>
+      <xdr:colOff>26516</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>26656</xdr:rowOff>
     </xdr:from>
@@ -4350,7 +4363,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="19539160" y="1972477"/>
+          <a:off x="26796302" y="2022370"/>
           <a:ext cx="1732998" cy="437873"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4413,7 +4426,7 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>47</xdr:col>
-      <xdr:colOff>53551</xdr:colOff>
+      <xdr:colOff>26336</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>179139</xdr:rowOff>
     </xdr:from>
@@ -4431,7 +4444,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="19445137" y="2754173"/>
+          <a:off x="26796122" y="2719139"/>
           <a:ext cx="1732998" cy="437873"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4494,13 +4507,13 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>48</xdr:col>
-      <xdr:colOff>318867</xdr:colOff>
+      <xdr:colOff>291541</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>154113</xdr:rowOff>
+      <xdr:rowOff>153675</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>48</xdr:col>
-      <xdr:colOff>319632</xdr:colOff>
+      <xdr:colOff>298941</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>87801</xdr:rowOff>
     </xdr:to>
@@ -4519,9 +4532,9 @@
         </xdr:cNvCxnSpPr>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
-        <a:xfrm>
-          <a:off x="20319177" y="1073768"/>
-          <a:ext cx="765" cy="301550"/>
+        <a:xfrm flipH="1">
+          <a:off x="27887894" y="1087499"/>
+          <a:ext cx="7400" cy="307655"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -4553,13 +4566,13 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>48</xdr:col>
-      <xdr:colOff>311506</xdr:colOff>
+      <xdr:colOff>285230</xdr:colOff>
       <xdr:row>8</xdr:row>
-      <xdr:rowOff>168430</xdr:rowOff>
+      <xdr:rowOff>170932</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>48</xdr:col>
-      <xdr:colOff>319632</xdr:colOff>
+      <xdr:colOff>293356</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>26656</xdr:rowOff>
     </xdr:to>
@@ -4579,8 +4592,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipH="1">
-          <a:off x="20311816" y="1639878"/>
-          <a:ext cx="8126" cy="410019"/>
+          <a:off x="27662801" y="1622361"/>
+          <a:ext cx="8126" cy="400009"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -4612,13 +4625,13 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>48</xdr:col>
-      <xdr:colOff>311326</xdr:colOff>
+      <xdr:colOff>285050</xdr:colOff>
       <xdr:row>13</xdr:row>
-      <xdr:rowOff>96667</xdr:rowOff>
+      <xdr:rowOff>101672</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>48</xdr:col>
-      <xdr:colOff>311506</xdr:colOff>
+      <xdr:colOff>285230</xdr:colOff>
       <xdr:row>14</xdr:row>
       <xdr:rowOff>179139</xdr:rowOff>
     </xdr:to>
@@ -4639,8 +4652,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipH="1">
-          <a:off x="20311636" y="2487770"/>
-          <a:ext cx="180" cy="266403"/>
+          <a:off x="27662621" y="2460243"/>
+          <a:ext cx="180" cy="258896"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -4753,13 +4766,13 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>48</xdr:col>
-      <xdr:colOff>311326</xdr:colOff>
+      <xdr:colOff>285050</xdr:colOff>
       <xdr:row>17</xdr:row>
-      <xdr:rowOff>65218</xdr:rowOff>
+      <xdr:rowOff>72726</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>48</xdr:col>
-      <xdr:colOff>312887</xdr:colOff>
+      <xdr:colOff>313826</xdr:colOff>
       <xdr:row>18</xdr:row>
       <xdr:rowOff>176493</xdr:rowOff>
     </xdr:to>
@@ -4780,8 +4793,8 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="20311636" y="3192046"/>
-          <a:ext cx="1561" cy="295206"/>
+          <a:off x="27662621" y="3157012"/>
+          <a:ext cx="28776" cy="285195"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -4955,7 +4968,7 @@
           <a:pPr algn="l"/>
           <a:r>
             <a:rPr lang="en-MY" sz="1100" b="0" u="none"/>
-            <a:t>-  assign by prediction score</a:t>
+            <a:t>-  Assign by prediction score</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -5241,7 +5254,7 @@
           <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="en-MY" sz="1100" b="0" u="none"/>
-            <a:t>floating cluster</a:t>
+            <a:t>Floating cluster</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -5497,7 +5510,7 @@
           <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="en-MY" sz="1100" b="0" u="none"/>
-            <a:t>Split KNOWN/UNKNOWN</a:t>
+            <a:t>Split Known/Unknown</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -5685,7 +5698,7 @@
           <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="en-MY" sz="1100" b="0" u="none"/>
-            <a:t>KNOWN</a:t>
+            <a:t>Known</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -5754,7 +5767,7 @@
           <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="en-MY" sz="1100" b="0" u="none"/>
-            <a:t>UNKNOWN</a:t>
+            <a:t>Unknown</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -6116,7 +6129,7 @@
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
-          <a:schemeClr val="accent5">
+          <a:schemeClr val="accent1">
             <a:lumMod val="20000"/>
             <a:lumOff val="80000"/>
           </a:schemeClr>
@@ -6454,7 +6467,7 @@
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
-          <a:schemeClr val="accent5">
+          <a:schemeClr val="accent1">
             <a:lumMod val="20000"/>
             <a:lumOff val="80000"/>
           </a:schemeClr>
@@ -6626,7 +6639,7 @@
           <a:pPr algn="ctr"/>
           <a:r>
             <a:rPr lang="en-MY"/>
-            <a:t>Update SQL MERGE </a:t>
+            <a:t>Update SQL</a:t>
           </a:r>
           <a:endParaRPr lang="en-MY" sz="1100" b="0" u="none"/>
         </a:p>
@@ -7341,6 +7354,858 @@
         </a:prstGeom>
       </xdr:spPr>
     </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>59</xdr:col>
+      <xdr:colOff>433773</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>122649</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1059934" cy="264560"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="31" name="TextBox 30">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{83E92520-E2E9-456E-B1C5-574C5758C5DE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="34469773" y="869708"/>
+          <a:ext cx="1059934" cy="264560"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent1">
+            <a:lumMod val="20000"/>
+            <a:lumOff val="80000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t">
+          <a:spAutoFit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-MY" sz="1100" b="0" u="none"/>
+            <a:t>Read Device ID</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>59</xdr:col>
+      <xdr:colOff>97241</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>58917</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1732998" cy="279558"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="35" name="TextBox 34">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{916A8FFB-6479-46B9-9283-92F1E4C37B88}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="34133241" y="1366270"/>
+          <a:ext cx="1732998" cy="279558"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent1">
+            <a:lumMod val="20000"/>
+            <a:lumOff val="80000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-MY" sz="1100" b="0" u="none"/>
+            <a:t>Predict Device</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-MY" sz="1100" b="0" u="none" baseline="0"/>
+            <a:t> Type </a:t>
+          </a:r>
+          <a:endParaRPr lang="en-MY" sz="1100" b="0" u="none"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>59</xdr:col>
+      <xdr:colOff>97241</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>6163</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1732998" cy="279558"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="43" name="TextBox 42">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{14DA3686-B724-4343-BE1E-A08B0095188A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="34133241" y="1873810"/>
+          <a:ext cx="1732998" cy="279558"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent1">
+            <a:lumMod val="20000"/>
+            <a:lumOff val="80000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-MY" sz="1100" b="0" u="none"/>
+            <a:t>Predict</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-MY" sz="1100" b="0" u="none" baseline="0"/>
+            <a:t> Section &amp; Cluster </a:t>
+          </a:r>
+          <a:endParaRPr lang="en-MY" sz="1100" b="0" u="none"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>59</xdr:col>
+      <xdr:colOff>97241</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>32715</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1732998" cy="279558"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="49" name="TextBox 48">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6952C101-EAF0-4A2D-B1ED-F4A4579EDC28}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="34133241" y="2460656"/>
+          <a:ext cx="1732998" cy="279558"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent1">
+            <a:lumMod val="20000"/>
+            <a:lumOff val="80000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-MY" sz="1100" b="0" u="none"/>
+            <a:t>Load Customer Quota</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>59</xdr:col>
+      <xdr:colOff>97241</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>111845</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1732998" cy="279558"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="53" name="TextBox 52">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{061D9418-DB2C-4160-9F9C-A18B8667DA70}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="34133241" y="2913316"/>
+          <a:ext cx="1732998" cy="279558"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent1">
+            <a:lumMod val="20000"/>
+            <a:lumOff val="80000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-MY" sz="1100" b="0" u="none"/>
+            <a:t>Allocate Devices</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>58</xdr:col>
+      <xdr:colOff>570737</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>63976</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2011182" cy="279558"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="55" name="TextBox 54">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5C48F08B-8802-4A3F-A640-9EF4552B4E6A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="33994149" y="3425741"/>
+          <a:ext cx="2011182" cy="279558"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent1">
+            <a:lumMod val="20000"/>
+            <a:lumOff val="80000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-MY" sz="1100" b="0" u="none"/>
+            <a:t>Separate Unassigned Devices</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>58</xdr:col>
+      <xdr:colOff>570737</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>177300</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="2011182" cy="279558"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="60" name="TextBox 59">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{57E728D5-F1F5-421B-A1AC-BECF7EC47795}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="33994149" y="3912594"/>
+          <a:ext cx="2011182" cy="279558"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent1">
+            <a:lumMod val="20000"/>
+            <a:lumOff val="80000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="en-MY" sz="1100" b="0" u="none"/>
+            <a:t>Write</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-MY" sz="1100" b="0" u="none" baseline="0"/>
+            <a:t> Result to SQL</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-MY" sz="1100" b="0" u="none"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>60</xdr:col>
+      <xdr:colOff>355016</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>19347</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>60</xdr:col>
+      <xdr:colOff>355016</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>58917</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="63" name="Straight Arrow Connector 62">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{919DDEB6-F3AC-4D1F-AA4E-7E22E5966230}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="31" idx="2"/>
+          <a:endCxn id="35" idx="0"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="34789533" y="1122933"/>
+          <a:ext cx="0" cy="223501"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="38100">
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>60</xdr:col>
+      <xdr:colOff>355016</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>154544</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>60</xdr:col>
+      <xdr:colOff>355016</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>6163</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="71" name="Straight Arrow Connector 70">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BCC5BCA2-49A5-46E4-B366-190300356F91}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="35" idx="2"/>
+          <a:endCxn id="43" idx="0"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="34789533" y="1625992"/>
+          <a:ext cx="0" cy="219481"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="38100">
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>60</xdr:col>
+      <xdr:colOff>355016</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>101790</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>60</xdr:col>
+      <xdr:colOff>355016</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>32715</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="85" name="Straight Arrow Connector 84">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4AFE7825-DD08-40B9-A8B2-707F8163362C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="43" idx="2"/>
+          <a:endCxn id="49" idx="0"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="34789533" y="2125031"/>
+          <a:ext cx="0" cy="298787"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="38100">
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>60</xdr:col>
+      <xdr:colOff>355016</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>128342</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>60</xdr:col>
+      <xdr:colOff>355016</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>111845</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="92" name="Straight Arrow Connector 91">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C45A1130-2401-41BF-ABF5-B722CF2F2892}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="49" idx="2"/>
+          <a:endCxn id="53" idx="0"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="34789533" y="2703376"/>
+          <a:ext cx="0" cy="167435"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="38100">
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>60</xdr:col>
+      <xdr:colOff>355016</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>23541</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>60</xdr:col>
+      <xdr:colOff>358880</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>63976</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="97" name="Straight Arrow Connector 96">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B63B7619-A30C-478E-93C5-1684DDDA7103}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="53" idx="2"/>
+          <a:endCxn id="55" idx="0"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="34789533" y="3150369"/>
+          <a:ext cx="3864" cy="224366"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="38100">
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>60</xdr:col>
+      <xdr:colOff>358880</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>159603</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>60</xdr:col>
+      <xdr:colOff>358880</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>177300</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="103" name="Straight Arrow Connector 102">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{56E77DD7-23A2-4AC9-95A1-619BFFB1E847}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:stCxn id="55" idx="2"/>
+          <a:endCxn id="60" idx="0"/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="34793397" y="3654293"/>
+          <a:ext cx="0" cy="201628"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="38100">
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -9216,7 +10081,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38AA77DD-8AB1-42B3-B673-04FA8231C115}">
-  <dimension ref="B2:BF84"/>
+  <dimension ref="B2:BS84"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="12" max="12" width="8.7265625" customWidth="1"/>
@@ -9228,174 +10093,1190 @@
     <col min="57" max="57" width="4.453125" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:58" x14ac:dyDescent="0.35">
-      <c r="B2" s="14" t="s">
+    <row r="2" spans="2:71" x14ac:dyDescent="0.35">
+      <c r="B2" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="14"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
+      <c r="J2" s="15"/>
+      <c r="K2" s="15"/>
       <c r="L2" s="13"/>
-      <c r="O2" s="14" t="s">
+      <c r="O2" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="P2" s="14"/>
-      <c r="Q2" s="14"/>
-      <c r="R2" s="14"/>
-      <c r="S2" s="14"/>
-      <c r="T2" s="14"/>
-      <c r="U2" s="14"/>
-      <c r="V2" s="14"/>
-      <c r="W2" s="14"/>
-      <c r="AA2" s="14" t="s">
+      <c r="P2" s="15"/>
+      <c r="Q2" s="15"/>
+      <c r="R2" s="15"/>
+      <c r="S2" s="15"/>
+      <c r="T2" s="15"/>
+      <c r="U2" s="15"/>
+      <c r="V2" s="15"/>
+      <c r="W2" s="15"/>
+      <c r="AA2" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="AB2" s="14"/>
-      <c r="AC2" s="14"/>
-      <c r="AD2" s="14"/>
-      <c r="AE2" s="14"/>
-      <c r="AI2" s="14" t="s">
+      <c r="AB2" s="15"/>
+      <c r="AC2" s="15"/>
+      <c r="AD2" s="15"/>
+      <c r="AE2" s="15"/>
+      <c r="AI2" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="AJ2" s="14"/>
-      <c r="AK2" s="14"/>
-      <c r="AL2" s="14"/>
-      <c r="AM2" s="14"/>
-      <c r="AQ2" s="14" t="s">
+      <c r="AJ2" s="15"/>
+      <c r="AK2" s="15"/>
+      <c r="AL2" s="15"/>
+      <c r="AM2" s="15"/>
+      <c r="AP2" s="10"/>
+      <c r="AQ2" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="AR2" s="14"/>
-      <c r="AS2" s="14"/>
-      <c r="AT2" s="14"/>
-      <c r="AU2" s="14"/>
-      <c r="AV2" s="14"/>
-      <c r="AW2" s="14"/>
-      <c r="AX2" s="14"/>
-      <c r="AY2" s="14"/>
-      <c r="AZ2" s="14"/>
-      <c r="BA2" s="14"/>
-      <c r="BB2" s="14"/>
-      <c r="BC2" s="14"/>
+      <c r="AR2" s="18"/>
+      <c r="AS2" s="18"/>
+      <c r="AT2" s="18"/>
+      <c r="AU2" s="18"/>
+      <c r="AV2" s="18"/>
+      <c r="AW2" s="18"/>
+      <c r="AX2" s="18"/>
+      <c r="AY2" s="18"/>
+      <c r="AZ2" s="18"/>
+      <c r="BA2" s="18"/>
+      <c r="BB2" s="18"/>
+      <c r="BC2" s="18"/>
       <c r="BD2" s="11"/>
       <c r="BE2" s="12"/>
       <c r="BF2" s="11"/>
+      <c r="BG2" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="BH2" s="18"/>
+      <c r="BI2" s="18"/>
+      <c r="BJ2" s="18"/>
+      <c r="BK2" s="18"/>
+      <c r="BL2" s="18"/>
+      <c r="BM2" s="19"/>
+      <c r="BN2" s="19"/>
+      <c r="BO2" s="19"/>
+      <c r="BP2" s="19"/>
+      <c r="BQ2" s="19"/>
+      <c r="BR2" s="19"/>
+      <c r="BS2" s="19"/>
     </row>
-    <row r="3" spans="2:58" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:71" x14ac:dyDescent="0.35">
+      <c r="AP3" s="10"/>
+      <c r="AQ3" s="10"/>
+      <c r="AR3" s="10"/>
+      <c r="AS3" s="10"/>
+      <c r="AT3" s="10"/>
+      <c r="AU3" s="10"/>
+      <c r="AV3" s="10"/>
+      <c r="AW3" s="10"/>
+      <c r="AX3" s="10"/>
+      <c r="AY3" s="10"/>
+      <c r="AZ3" s="10"/>
+      <c r="BA3" s="10"/>
+      <c r="BB3" s="10"/>
       <c r="BC3" s="10"/>
+      <c r="BD3" s="10"/>
     </row>
-    <row r="15" spans="2:58" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:71" x14ac:dyDescent="0.35">
+      <c r="AP4" s="10"/>
+      <c r="AQ4" s="10"/>
+      <c r="AR4" s="10"/>
+      <c r="AS4" s="10"/>
+      <c r="AT4" s="10"/>
+      <c r="AU4" s="10"/>
+      <c r="AV4" s="10"/>
+      <c r="AW4" s="10"/>
+      <c r="AX4" s="10"/>
+      <c r="AY4" s="10"/>
+      <c r="AZ4" s="10"/>
+      <c r="BA4" s="10"/>
+      <c r="BB4" s="10"/>
+      <c r="BC4" s="10"/>
+      <c r="BD4" s="10"/>
+    </row>
+    <row r="5" spans="2:71" x14ac:dyDescent="0.35">
+      <c r="AP5" s="10"/>
+      <c r="AQ5" s="10"/>
+      <c r="AR5" s="10"/>
+      <c r="AS5" s="10"/>
+      <c r="AT5" s="10"/>
+      <c r="AU5" s="10"/>
+      <c r="AV5" s="10"/>
+      <c r="AW5" s="10"/>
+      <c r="AX5" s="10"/>
+      <c r="AY5" s="10"/>
+      <c r="AZ5" s="10"/>
+      <c r="BA5" s="10"/>
+      <c r="BB5" s="10"/>
+      <c r="BC5" s="10"/>
+      <c r="BD5" s="10"/>
+    </row>
+    <row r="6" spans="2:71" x14ac:dyDescent="0.35">
+      <c r="AP6" s="10"/>
+      <c r="AQ6" s="10"/>
+      <c r="AR6" s="10"/>
+      <c r="AS6" s="10"/>
+      <c r="AT6" s="10"/>
+      <c r="AU6" s="10"/>
+      <c r="AV6" s="10"/>
+      <c r="AW6" s="10"/>
+      <c r="AX6" s="10"/>
+      <c r="AY6" s="10"/>
+      <c r="AZ6" s="10"/>
+      <c r="BA6" s="10"/>
+      <c r="BB6" s="10"/>
+      <c r="BC6" s="10"/>
+      <c r="BD6" s="10"/>
+    </row>
+    <row r="7" spans="2:71" x14ac:dyDescent="0.35">
+      <c r="AP7" s="10"/>
+      <c r="AQ7" s="10"/>
+      <c r="AR7" s="10"/>
+      <c r="AS7" s="10"/>
+      <c r="AT7" s="10"/>
+      <c r="AU7" s="10"/>
+      <c r="AV7" s="10"/>
+      <c r="AW7" s="10"/>
+      <c r="AX7" s="10"/>
+      <c r="AY7" s="10"/>
+      <c r="AZ7" s="10"/>
+      <c r="BA7" s="10"/>
+      <c r="BB7" s="10"/>
+      <c r="BC7" s="10"/>
+      <c r="BD7" s="10"/>
+    </row>
+    <row r="8" spans="2:71" x14ac:dyDescent="0.35">
+      <c r="AP8" s="10"/>
+      <c r="AQ8" s="10"/>
+      <c r="AR8" s="10"/>
+      <c r="AS8" s="10"/>
+      <c r="AT8" s="10"/>
+      <c r="AU8" s="10"/>
+      <c r="AV8" s="10"/>
+      <c r="AW8" s="10"/>
+      <c r="AX8" s="10"/>
+      <c r="AY8" s="10"/>
+      <c r="AZ8" s="10"/>
+      <c r="BA8" s="10"/>
+      <c r="BB8" s="10"/>
+      <c r="BC8" s="10"/>
+      <c r="BD8" s="10"/>
+    </row>
+    <row r="9" spans="2:71" x14ac:dyDescent="0.35">
+      <c r="AP9" s="10"/>
+      <c r="AQ9" s="10"/>
+      <c r="AR9" s="10"/>
+      <c r="AS9" s="10"/>
+      <c r="AT9" s="10"/>
+      <c r="AU9" s="10"/>
+      <c r="AV9" s="10"/>
+      <c r="AW9" s="10"/>
+      <c r="AX9" s="10"/>
+      <c r="AY9" s="10"/>
+      <c r="AZ9" s="10"/>
+      <c r="BA9" s="10"/>
+      <c r="BB9" s="10"/>
+      <c r="BC9" s="10"/>
+      <c r="BD9" s="10"/>
+    </row>
+    <row r="10" spans="2:71" x14ac:dyDescent="0.35">
+      <c r="AP10" s="10"/>
+      <c r="AQ10" s="10"/>
+      <c r="AR10" s="10"/>
+      <c r="AS10" s="10"/>
+      <c r="AT10" s="10"/>
+      <c r="AU10" s="10"/>
+      <c r="AV10" s="10"/>
+      <c r="AW10" s="10"/>
+      <c r="AX10" s="10"/>
+      <c r="AY10" s="10"/>
+      <c r="AZ10" s="10"/>
+      <c r="BA10" s="10"/>
+      <c r="BB10" s="10"/>
+      <c r="BC10" s="10"/>
+      <c r="BD10" s="10"/>
+    </row>
+    <row r="11" spans="2:71" x14ac:dyDescent="0.35">
+      <c r="AP11" s="10"/>
+      <c r="AQ11" s="10"/>
+      <c r="AR11" s="10"/>
+      <c r="AS11" s="10"/>
+      <c r="AT11" s="10"/>
+      <c r="AU11" s="10"/>
+      <c r="AV11" s="10"/>
+      <c r="AW11" s="10"/>
+      <c r="AX11" s="10"/>
+      <c r="AY11" s="10"/>
+      <c r="AZ11" s="10"/>
+      <c r="BA11" s="10"/>
+      <c r="BB11" s="10"/>
+      <c r="BC11" s="10"/>
+      <c r="BD11" s="10"/>
+    </row>
+    <row r="12" spans="2:71" x14ac:dyDescent="0.35">
+      <c r="AP12" s="10"/>
+      <c r="AQ12" s="10"/>
+      <c r="AR12" s="10"/>
+      <c r="AS12" s="10"/>
+      <c r="AT12" s="10"/>
+      <c r="AU12" s="10"/>
+      <c r="AV12" s="10"/>
+      <c r="AW12" s="10"/>
+      <c r="AX12" s="10"/>
+      <c r="AY12" s="10"/>
+      <c r="AZ12" s="10"/>
+      <c r="BA12" s="10"/>
+      <c r="BB12" s="10"/>
+      <c r="BC12" s="10"/>
+      <c r="BD12" s="10"/>
+    </row>
+    <row r="13" spans="2:71" x14ac:dyDescent="0.35">
+      <c r="AP13" s="10"/>
+      <c r="AQ13" s="10"/>
+      <c r="AR13" s="10"/>
+      <c r="AS13" s="10"/>
+      <c r="AT13" s="10"/>
+      <c r="AU13" s="10"/>
+      <c r="AV13" s="10"/>
+      <c r="AW13" s="10"/>
+      <c r="AX13" s="10"/>
+      <c r="AY13" s="10"/>
+      <c r="AZ13" s="10"/>
+      <c r="BA13" s="10"/>
+      <c r="BB13" s="10"/>
+      <c r="BC13" s="10"/>
+      <c r="BD13" s="10"/>
+    </row>
+    <row r="14" spans="2:71" x14ac:dyDescent="0.35">
+      <c r="AP14" s="10"/>
+      <c r="AQ14" s="10"/>
+      <c r="AR14" s="10"/>
+      <c r="AS14" s="10"/>
+      <c r="AT14" s="10"/>
+      <c r="AU14" s="10"/>
+      <c r="AV14" s="10"/>
+      <c r="AW14" s="10"/>
+      <c r="AX14" s="10"/>
+      <c r="AY14" s="10"/>
+      <c r="AZ14" s="10"/>
+      <c r="BA14" s="10"/>
+      <c r="BB14" s="10"/>
+      <c r="BC14" s="10"/>
+      <c r="BD14" s="10"/>
+    </row>
+    <row r="15" spans="2:71" x14ac:dyDescent="0.35">
       <c r="T15" s="1"/>
+      <c r="AP15" s="10"/>
+      <c r="AQ15" s="10"/>
+      <c r="AR15" s="10"/>
+      <c r="AS15" s="10"/>
+      <c r="AT15" s="10"/>
+      <c r="AU15" s="10"/>
+      <c r="AV15" s="10"/>
+      <c r="AW15" s="10"/>
+      <c r="AX15" s="10"/>
+      <c r="AY15" s="10"/>
+      <c r="AZ15" s="10"/>
+      <c r="BA15" s="10"/>
+      <c r="BB15" s="10"/>
+      <c r="BC15" s="10"/>
+      <c r="BD15" s="10"/>
     </row>
-    <row r="43" spans="15:36" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:71" x14ac:dyDescent="0.35">
+      <c r="AP16" s="10"/>
+      <c r="AQ16" s="10"/>
+      <c r="AR16" s="10"/>
+      <c r="AS16" s="10"/>
+      <c r="AT16" s="10"/>
+      <c r="AU16" s="10"/>
+      <c r="AV16" s="10"/>
+      <c r="AW16" s="10"/>
+      <c r="AX16" s="10"/>
+      <c r="AY16" s="10"/>
+      <c r="AZ16" s="10"/>
+      <c r="BA16" s="10"/>
+      <c r="BB16" s="10"/>
+      <c r="BC16" s="10"/>
+      <c r="BD16" s="10"/>
+    </row>
+    <row r="17" spans="42:56" x14ac:dyDescent="0.35">
+      <c r="AP17" s="10"/>
+      <c r="AQ17" s="10"/>
+      <c r="AR17" s="10"/>
+      <c r="AS17" s="10"/>
+      <c r="AT17" s="10"/>
+      <c r="AU17" s="10"/>
+      <c r="AV17" s="10"/>
+      <c r="AW17" s="10"/>
+      <c r="AX17" s="10"/>
+      <c r="AY17" s="10"/>
+      <c r="AZ17" s="10"/>
+      <c r="BA17" s="10"/>
+      <c r="BB17" s="10"/>
+      <c r="BC17" s="10"/>
+      <c r="BD17" s="10"/>
+    </row>
+    <row r="18" spans="42:56" x14ac:dyDescent="0.35">
+      <c r="AP18" s="10"/>
+      <c r="AQ18" s="10"/>
+      <c r="AR18" s="10"/>
+      <c r="AS18" s="10"/>
+      <c r="AT18" s="10"/>
+      <c r="AU18" s="10"/>
+      <c r="AV18" s="10"/>
+      <c r="AW18" s="10"/>
+      <c r="AX18" s="10"/>
+      <c r="AY18" s="10"/>
+      <c r="AZ18" s="10"/>
+      <c r="BA18" s="10"/>
+      <c r="BB18" s="10"/>
+      <c r="BC18" s="10"/>
+      <c r="BD18" s="10"/>
+    </row>
+    <row r="19" spans="42:56" x14ac:dyDescent="0.35">
+      <c r="AP19" s="10"/>
+      <c r="AQ19" s="10"/>
+      <c r="AR19" s="10"/>
+      <c r="AS19" s="10"/>
+      <c r="AT19" s="10"/>
+      <c r="AU19" s="10"/>
+      <c r="AV19" s="10"/>
+      <c r="AW19" s="10"/>
+      <c r="AX19" s="10"/>
+      <c r="AY19" s="10"/>
+      <c r="AZ19" s="10"/>
+      <c r="BA19" s="10"/>
+      <c r="BB19" s="10"/>
+      <c r="BC19" s="10"/>
+      <c r="BD19" s="10"/>
+    </row>
+    <row r="20" spans="42:56" x14ac:dyDescent="0.35">
+      <c r="AP20" s="10"/>
+      <c r="AQ20" s="10"/>
+      <c r="AR20" s="10"/>
+      <c r="AS20" s="10"/>
+      <c r="AT20" s="10"/>
+      <c r="AU20" s="10"/>
+      <c r="AV20" s="10"/>
+      <c r="AW20" s="10"/>
+      <c r="AX20" s="10"/>
+      <c r="AY20" s="10"/>
+      <c r="AZ20" s="10"/>
+      <c r="BA20" s="10"/>
+      <c r="BB20" s="10"/>
+      <c r="BC20" s="10"/>
+      <c r="BD20" s="10"/>
+    </row>
+    <row r="21" spans="42:56" x14ac:dyDescent="0.35">
+      <c r="AP21" s="10"/>
+      <c r="AQ21" s="10"/>
+      <c r="AR21" s="10"/>
+      <c r="AS21" s="10"/>
+      <c r="AT21" s="10"/>
+      <c r="AU21" s="10"/>
+      <c r="AV21" s="10"/>
+      <c r="AW21" s="10"/>
+      <c r="AX21" s="10"/>
+      <c r="AY21" s="10"/>
+      <c r="AZ21" s="10"/>
+      <c r="BA21" s="10"/>
+      <c r="BB21" s="10"/>
+      <c r="BC21" s="10"/>
+      <c r="BD21" s="10"/>
+    </row>
+    <row r="22" spans="42:56" x14ac:dyDescent="0.35">
+      <c r="AP22" s="10"/>
+      <c r="AQ22" s="10"/>
+      <c r="AR22" s="10"/>
+      <c r="AS22" s="10"/>
+      <c r="AT22" s="10"/>
+      <c r="AU22" s="10"/>
+      <c r="AV22" s="10"/>
+      <c r="AW22" s="10"/>
+      <c r="AX22" s="10"/>
+      <c r="AY22" s="10"/>
+      <c r="AZ22" s="10"/>
+      <c r="BA22" s="10"/>
+      <c r="BB22" s="10"/>
+      <c r="BC22" s="10"/>
+      <c r="BD22" s="10"/>
+    </row>
+    <row r="23" spans="42:56" x14ac:dyDescent="0.35">
+      <c r="AP23" s="10"/>
+      <c r="AQ23" s="10"/>
+      <c r="AR23" s="10"/>
+      <c r="AS23" s="10"/>
+      <c r="AT23" s="10"/>
+      <c r="AU23" s="10"/>
+      <c r="AV23" s="10"/>
+      <c r="AW23" s="10"/>
+      <c r="AX23" s="10"/>
+      <c r="AY23" s="10"/>
+      <c r="AZ23" s="10"/>
+      <c r="BA23" s="10"/>
+      <c r="BB23" s="10"/>
+      <c r="BC23" s="10"/>
+      <c r="BD23" s="10"/>
+    </row>
+    <row r="24" spans="42:56" x14ac:dyDescent="0.35">
+      <c r="AP24" s="10"/>
+      <c r="AQ24" s="10"/>
+      <c r="AR24" s="10"/>
+      <c r="AS24" s="10"/>
+      <c r="AT24" s="10"/>
+      <c r="AU24" s="10"/>
+      <c r="AV24" s="10"/>
+      <c r="AW24" s="10"/>
+      <c r="AX24" s="10"/>
+      <c r="AY24" s="10"/>
+      <c r="AZ24" s="10"/>
+      <c r="BA24" s="10"/>
+      <c r="BB24" s="10"/>
+      <c r="BC24" s="10"/>
+      <c r="BD24" s="10"/>
+    </row>
+    <row r="25" spans="42:56" x14ac:dyDescent="0.35">
+      <c r="AP25" s="10"/>
+      <c r="AQ25" s="10"/>
+      <c r="AR25" s="10"/>
+      <c r="AS25" s="10"/>
+      <c r="AT25" s="10"/>
+      <c r="AU25" s="10"/>
+      <c r="AV25" s="10"/>
+      <c r="AW25" s="10"/>
+      <c r="AX25" s="10"/>
+      <c r="AY25" s="10"/>
+      <c r="AZ25" s="10"/>
+      <c r="BA25" s="10"/>
+      <c r="BB25" s="10"/>
+      <c r="BC25" s="10"/>
+      <c r="BD25" s="10"/>
+    </row>
+    <row r="26" spans="42:56" x14ac:dyDescent="0.35">
+      <c r="AP26" s="10"/>
+      <c r="AQ26" s="10"/>
+      <c r="AR26" s="10"/>
+      <c r="AS26" s="10"/>
+      <c r="AT26" s="10"/>
+      <c r="AU26" s="10"/>
+      <c r="AV26" s="10"/>
+      <c r="AW26" s="10"/>
+      <c r="AX26" s="10"/>
+      <c r="AY26" s="10"/>
+      <c r="AZ26" s="10"/>
+      <c r="BA26" s="10"/>
+      <c r="BB26" s="10"/>
+      <c r="BC26" s="10"/>
+      <c r="BD26" s="10"/>
+    </row>
+    <row r="27" spans="42:56" x14ac:dyDescent="0.35">
+      <c r="AP27" s="10"/>
+      <c r="AQ27" s="10"/>
+      <c r="AR27" s="10"/>
+      <c r="AS27" s="10"/>
+      <c r="AT27" s="10"/>
+      <c r="AU27" s="10"/>
+      <c r="AV27" s="10"/>
+      <c r="AW27" s="10"/>
+      <c r="AX27" s="10"/>
+      <c r="AY27" s="10"/>
+      <c r="AZ27" s="10"/>
+      <c r="BA27" s="10"/>
+      <c r="BB27" s="10"/>
+      <c r="BC27" s="10"/>
+      <c r="BD27" s="10"/>
+    </row>
+    <row r="28" spans="42:56" x14ac:dyDescent="0.35">
+      <c r="AP28" s="10"/>
+      <c r="AQ28" s="10"/>
+      <c r="AR28" s="10"/>
+      <c r="AS28" s="10"/>
+      <c r="AT28" s="10"/>
+      <c r="AU28" s="10"/>
+      <c r="AV28" s="10"/>
+      <c r="AW28" s="10"/>
+      <c r="AX28" s="10"/>
+      <c r="AY28" s="10"/>
+      <c r="AZ28" s="10"/>
+      <c r="BA28" s="10"/>
+      <c r="BB28" s="10"/>
+      <c r="BC28" s="10"/>
+      <c r="BD28" s="10"/>
+    </row>
+    <row r="29" spans="42:56" x14ac:dyDescent="0.35">
+      <c r="AP29" s="10"/>
+      <c r="AQ29" s="10"/>
+      <c r="AR29" s="10"/>
+      <c r="AS29" s="10"/>
+      <c r="AT29" s="10"/>
+      <c r="AU29" s="10"/>
+      <c r="AV29" s="10"/>
+      <c r="AW29" s="10"/>
+      <c r="AX29" s="10"/>
+      <c r="AY29" s="10"/>
+      <c r="AZ29" s="10"/>
+      <c r="BA29" s="10"/>
+      <c r="BB29" s="10"/>
+      <c r="BC29" s="10"/>
+      <c r="BD29" s="10"/>
+    </row>
+    <row r="30" spans="42:56" x14ac:dyDescent="0.35">
+      <c r="AP30" s="10"/>
+      <c r="AQ30" s="10"/>
+      <c r="AR30" s="10"/>
+      <c r="AS30" s="10"/>
+      <c r="AT30" s="10"/>
+      <c r="AU30" s="10"/>
+      <c r="AV30" s="10"/>
+      <c r="AW30" s="10"/>
+      <c r="AX30" s="10"/>
+      <c r="AY30" s="10"/>
+      <c r="AZ30" s="10"/>
+      <c r="BA30" s="10"/>
+      <c r="BB30" s="10"/>
+      <c r="BC30" s="10"/>
+      <c r="BD30" s="10"/>
+    </row>
+    <row r="31" spans="42:56" x14ac:dyDescent="0.35">
+      <c r="AP31" s="10"/>
+      <c r="AQ31" s="10"/>
+      <c r="AR31" s="10"/>
+      <c r="AS31" s="10"/>
+      <c r="AT31" s="10"/>
+      <c r="AU31" s="10"/>
+      <c r="AV31" s="10"/>
+      <c r="AW31" s="10"/>
+      <c r="AX31" s="10"/>
+      <c r="AY31" s="10"/>
+      <c r="AZ31" s="10"/>
+      <c r="BA31" s="10"/>
+      <c r="BB31" s="10"/>
+      <c r="BC31" s="10"/>
+      <c r="BD31" s="10"/>
+    </row>
+    <row r="32" spans="42:56" x14ac:dyDescent="0.35">
+      <c r="AP32" s="10"/>
+      <c r="AQ32" s="10"/>
+      <c r="AR32" s="10"/>
+      <c r="AS32" s="10"/>
+      <c r="AT32" s="10"/>
+      <c r="AU32" s="10"/>
+      <c r="AV32" s="10"/>
+      <c r="AW32" s="10"/>
+      <c r="AX32" s="10"/>
+      <c r="AY32" s="10"/>
+      <c r="AZ32" s="10"/>
+      <c r="BA32" s="10"/>
+      <c r="BB32" s="10"/>
+      <c r="BC32" s="10"/>
+      <c r="BD32" s="10"/>
+    </row>
+    <row r="33" spans="15:56" x14ac:dyDescent="0.35">
+      <c r="AP33" s="10"/>
+      <c r="AQ33" s="10"/>
+      <c r="AR33" s="10"/>
+      <c r="AS33" s="10"/>
+      <c r="AT33" s="10"/>
+      <c r="AU33" s="10"/>
+      <c r="AV33" s="10"/>
+      <c r="AW33" s="10"/>
+      <c r="AX33" s="10"/>
+      <c r="AY33" s="10"/>
+      <c r="AZ33" s="10"/>
+      <c r="BA33" s="10"/>
+      <c r="BB33" s="10"/>
+      <c r="BC33" s="10"/>
+      <c r="BD33" s="10"/>
+    </row>
+    <row r="34" spans="15:56" x14ac:dyDescent="0.35">
+      <c r="AP34" s="10"/>
+      <c r="AQ34" s="10"/>
+      <c r="AR34" s="10"/>
+      <c r="AS34" s="10"/>
+      <c r="AT34" s="10"/>
+      <c r="AU34" s="10"/>
+      <c r="AV34" s="10"/>
+      <c r="AW34" s="10"/>
+      <c r="AX34" s="10"/>
+      <c r="AY34" s="10"/>
+      <c r="AZ34" s="10"/>
+      <c r="BA34" s="10"/>
+      <c r="BB34" s="10"/>
+      <c r="BC34" s="10"/>
+      <c r="BD34" s="10"/>
+    </row>
+    <row r="35" spans="15:56" x14ac:dyDescent="0.35">
+      <c r="AP35" s="10"/>
+      <c r="AQ35" s="10"/>
+      <c r="AR35" s="10"/>
+      <c r="AS35" s="10"/>
+      <c r="AT35" s="10"/>
+      <c r="AU35" s="10"/>
+      <c r="AV35" s="10"/>
+      <c r="AW35" s="10"/>
+      <c r="AX35" s="10"/>
+      <c r="AY35" s="10"/>
+      <c r="AZ35" s="10"/>
+      <c r="BA35" s="10"/>
+      <c r="BB35" s="10"/>
+      <c r="BC35" s="10"/>
+      <c r="BD35" s="10"/>
+    </row>
+    <row r="36" spans="15:56" x14ac:dyDescent="0.35">
+      <c r="AP36" s="10"/>
+      <c r="AQ36" s="10"/>
+      <c r="AR36" s="10"/>
+      <c r="AS36" s="10"/>
+      <c r="AT36" s="10"/>
+      <c r="AU36" s="10"/>
+      <c r="AV36" s="10"/>
+      <c r="AW36" s="10"/>
+      <c r="AX36" s="10"/>
+      <c r="AY36" s="10"/>
+      <c r="AZ36" s="10"/>
+      <c r="BA36" s="10"/>
+      <c r="BB36" s="10"/>
+      <c r="BC36" s="10"/>
+      <c r="BD36" s="10"/>
+    </row>
+    <row r="37" spans="15:56" x14ac:dyDescent="0.35">
+      <c r="AP37" s="10"/>
+      <c r="AQ37" s="10"/>
+      <c r="AR37" s="10"/>
+      <c r="AS37" s="10"/>
+      <c r="AT37" s="10"/>
+      <c r="AU37" s="10"/>
+      <c r="AV37" s="10"/>
+      <c r="AW37" s="10"/>
+      <c r="AX37" s="10"/>
+      <c r="AY37" s="10"/>
+      <c r="AZ37" s="10"/>
+      <c r="BA37" s="10"/>
+      <c r="BB37" s="10"/>
+      <c r="BC37" s="10"/>
+      <c r="BD37" s="10"/>
+    </row>
+    <row r="38" spans="15:56" x14ac:dyDescent="0.35">
+      <c r="AP38" s="10"/>
+      <c r="AQ38" s="10"/>
+      <c r="AR38" s="10"/>
+      <c r="AS38" s="10"/>
+      <c r="AT38" s="10"/>
+      <c r="AU38" s="10"/>
+      <c r="AV38" s="10"/>
+      <c r="AW38" s="10"/>
+      <c r="AX38" s="10"/>
+      <c r="AY38" s="10"/>
+      <c r="AZ38" s="10"/>
+      <c r="BA38" s="10"/>
+      <c r="BB38" s="10"/>
+      <c r="BC38" s="10"/>
+      <c r="BD38" s="10"/>
+    </row>
+    <row r="39" spans="15:56" x14ac:dyDescent="0.35">
+      <c r="AP39" s="10"/>
+      <c r="AQ39" s="10"/>
+      <c r="AR39" s="10"/>
+      <c r="AS39" s="10"/>
+      <c r="AT39" s="10"/>
+      <c r="AU39" s="10"/>
+      <c r="AV39" s="10"/>
+      <c r="AW39" s="10"/>
+      <c r="AX39" s="10"/>
+      <c r="AY39" s="10"/>
+      <c r="AZ39" s="10"/>
+      <c r="BA39" s="10"/>
+      <c r="BB39" s="10"/>
+      <c r="BC39" s="10"/>
+      <c r="BD39" s="10"/>
+    </row>
+    <row r="40" spans="15:56" x14ac:dyDescent="0.35">
+      <c r="AP40" s="10"/>
+      <c r="AQ40" s="10"/>
+      <c r="AR40" s="10"/>
+      <c r="AS40" s="10"/>
+      <c r="AT40" s="10"/>
+      <c r="AU40" s="10"/>
+      <c r="AV40" s="10"/>
+      <c r="AW40" s="10"/>
+      <c r="AX40" s="10"/>
+      <c r="AY40" s="10"/>
+      <c r="AZ40" s="10"/>
+      <c r="BA40" s="10"/>
+      <c r="BB40" s="10"/>
+      <c r="BC40" s="10"/>
+      <c r="BD40" s="10"/>
+    </row>
+    <row r="41" spans="15:56" x14ac:dyDescent="0.35">
+      <c r="AP41" s="10"/>
+      <c r="AQ41" s="10"/>
+      <c r="AR41" s="10"/>
+      <c r="AS41" s="10"/>
+      <c r="AT41" s="10"/>
+      <c r="AU41" s="10"/>
+      <c r="AV41" s="10"/>
+      <c r="AW41" s="10"/>
+      <c r="AX41" s="10"/>
+      <c r="AY41" s="10"/>
+      <c r="AZ41" s="10"/>
+      <c r="BA41" s="10"/>
+      <c r="BB41" s="10"/>
+      <c r="BC41" s="10"/>
+      <c r="BD41" s="10"/>
+    </row>
+    <row r="42" spans="15:56" x14ac:dyDescent="0.35">
+      <c r="AP42" s="10"/>
+      <c r="AQ42" s="10"/>
+      <c r="AR42" s="10"/>
+      <c r="AS42" s="10"/>
+      <c r="AT42" s="10"/>
+      <c r="AU42" s="10"/>
+      <c r="AV42" s="10"/>
+      <c r="AW42" s="10"/>
+      <c r="AX42" s="10"/>
+      <c r="AY42" s="10"/>
+      <c r="AZ42" s="10"/>
+      <c r="BA42" s="10"/>
+      <c r="BB42" s="10"/>
+      <c r="BC42" s="10"/>
+      <c r="BD42" s="10"/>
+    </row>
+    <row r="43" spans="15:56" x14ac:dyDescent="0.35">
       <c r="AJ43" t="s">
         <v>79</v>
       </c>
+      <c r="AP43" s="10"/>
+      <c r="AQ43" s="10"/>
+      <c r="AR43" s="10"/>
+      <c r="AS43" s="10"/>
+      <c r="AT43" s="10"/>
+      <c r="AU43" s="10"/>
+      <c r="AV43" s="10"/>
+      <c r="AW43" s="10"/>
+      <c r="AX43" s="10"/>
+      <c r="AY43" s="10"/>
+      <c r="AZ43" s="10"/>
+      <c r="BA43" s="10"/>
+      <c r="BB43" s="10"/>
+      <c r="BC43" s="10"/>
+      <c r="BD43" s="10"/>
     </row>
-    <row r="44" spans="15:36" x14ac:dyDescent="0.35">
+    <row r="44" spans="15:56" x14ac:dyDescent="0.35">
       <c r="AJ44" t="s">
         <v>78</v>
       </c>
+      <c r="AP44" s="10"/>
+      <c r="AQ44" s="10"/>
+      <c r="AR44" s="10"/>
+      <c r="AS44" s="10"/>
+      <c r="AT44" s="10"/>
+      <c r="AU44" s="10"/>
+      <c r="AV44" s="10"/>
+      <c r="AW44" s="10"/>
+      <c r="AX44" s="10"/>
+      <c r="AY44" s="10"/>
+      <c r="AZ44" s="10"/>
+      <c r="BA44" s="10"/>
+      <c r="BB44" s="10"/>
+      <c r="BC44" s="10"/>
+      <c r="BD44" s="10"/>
     </row>
-    <row r="48" spans="15:36" x14ac:dyDescent="0.35">
+    <row r="45" spans="15:56" x14ac:dyDescent="0.35">
+      <c r="AP45" s="10"/>
+      <c r="AQ45" s="10"/>
+      <c r="AR45" s="10"/>
+      <c r="AS45" s="10"/>
+      <c r="AT45" s="10"/>
+      <c r="AU45" s="10"/>
+      <c r="AV45" s="10"/>
+      <c r="AW45" s="10"/>
+      <c r="AX45" s="10"/>
+      <c r="AY45" s="10"/>
+      <c r="AZ45" s="10"/>
+      <c r="BA45" s="10"/>
+      <c r="BB45" s="10"/>
+      <c r="BC45" s="10"/>
+      <c r="BD45" s="10"/>
+    </row>
+    <row r="46" spans="15:56" x14ac:dyDescent="0.35">
+      <c r="AP46" s="10"/>
+      <c r="AQ46" s="10"/>
+      <c r="AR46" s="10"/>
+      <c r="AS46" s="10"/>
+      <c r="AT46" s="10"/>
+      <c r="AU46" s="10"/>
+      <c r="AV46" s="10"/>
+      <c r="AW46" s="10"/>
+      <c r="AX46" s="10"/>
+      <c r="AY46" s="10"/>
+      <c r="AZ46" s="10"/>
+      <c r="BA46" s="10"/>
+      <c r="BB46" s="10"/>
+      <c r="BC46" s="10"/>
+      <c r="BD46" s="10"/>
+    </row>
+    <row r="47" spans="15:56" x14ac:dyDescent="0.35">
+      <c r="AP47" s="10"/>
+      <c r="AQ47" s="10"/>
+      <c r="AR47" s="10"/>
+      <c r="AS47" s="10"/>
+      <c r="AT47" s="10"/>
+      <c r="AU47" s="10"/>
+      <c r="AV47" s="10"/>
+      <c r="AW47" s="10"/>
+      <c r="AX47" s="10"/>
+      <c r="AY47" s="10"/>
+      <c r="AZ47" s="10"/>
+      <c r="BA47" s="10"/>
+      <c r="BB47" s="10"/>
+      <c r="BC47" s="10"/>
+      <c r="BD47" s="10"/>
+    </row>
+    <row r="48" spans="15:56" x14ac:dyDescent="0.35">
       <c r="O48" s="16" t="s">
         <v>5</v>
       </c>
       <c r="P48" s="16"/>
       <c r="Q48" s="16"/>
       <c r="R48" s="16"/>
+      <c r="AP48" s="10"/>
+      <c r="AQ48" s="10"/>
+      <c r="AR48" s="10"/>
+      <c r="AS48" s="10"/>
+      <c r="AT48" s="10"/>
+      <c r="AU48" s="10"/>
+      <c r="AV48" s="10"/>
+      <c r="AW48" s="10"/>
+      <c r="AX48" s="10"/>
+      <c r="AY48" s="10"/>
+      <c r="AZ48" s="10"/>
+      <c r="BA48" s="10"/>
+      <c r="BB48" s="10"/>
+      <c r="BC48" s="10"/>
+      <c r="BD48" s="10"/>
     </row>
-    <row r="50" spans="27:39" x14ac:dyDescent="0.35">
-      <c r="AA50" s="15" t="s">
+    <row r="49" spans="27:56" x14ac:dyDescent="0.35">
+      <c r="AP49" s="10"/>
+      <c r="AQ49" s="10"/>
+      <c r="AR49" s="10"/>
+      <c r="AS49" s="10"/>
+      <c r="AT49" s="10"/>
+      <c r="AU49" s="10"/>
+      <c r="AV49" s="10"/>
+      <c r="AW49" s="10"/>
+      <c r="AX49" s="10"/>
+      <c r="AY49" s="10"/>
+      <c r="AZ49" s="10"/>
+      <c r="BA49" s="10"/>
+      <c r="BB49" s="10"/>
+      <c r="BC49" s="10"/>
+      <c r="BD49" s="10"/>
+    </row>
+    <row r="50" spans="27:56" x14ac:dyDescent="0.35">
+      <c r="AA50" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="AB50" s="15"/>
-      <c r="AC50" s="15"/>
-      <c r="AD50" s="15"/>
-      <c r="AE50" s="15"/>
+      <c r="AB50" s="14"/>
+      <c r="AC50" s="14"/>
+      <c r="AD50" s="14"/>
+      <c r="AE50" s="14"/>
       <c r="AI50" t="s">
         <v>80</v>
       </c>
+      <c r="AP50" s="10"/>
+      <c r="AQ50" s="10"/>
+      <c r="AR50" s="10"/>
+      <c r="AS50" s="10"/>
+      <c r="AT50" s="10"/>
+      <c r="AU50" s="10"/>
+      <c r="AV50" s="10"/>
+      <c r="AW50" s="10"/>
+      <c r="AX50" s="10"/>
+      <c r="AY50" s="10"/>
+      <c r="AZ50" s="10"/>
+      <c r="BA50" s="10"/>
+      <c r="BB50" s="10"/>
+      <c r="BC50" s="10"/>
+      <c r="BD50" s="10"/>
     </row>
-    <row r="51" spans="27:39" x14ac:dyDescent="0.35">
+    <row r="51" spans="27:56" x14ac:dyDescent="0.35">
       <c r="AI51" t="s">
         <v>81</v>
       </c>
+      <c r="AP51" s="10"/>
+      <c r="AQ51" s="10"/>
+      <c r="AR51" s="10"/>
+      <c r="AS51" s="10"/>
+      <c r="AT51" s="10"/>
+      <c r="AU51" s="10"/>
+      <c r="AV51" s="10"/>
+      <c r="AW51" s="10"/>
+      <c r="AX51" s="10"/>
+      <c r="AY51" s="10"/>
+      <c r="AZ51" s="10"/>
+      <c r="BA51" s="10"/>
+      <c r="BB51" s="10"/>
+      <c r="BC51" s="10"/>
+      <c r="BD51" s="10"/>
     </row>
-    <row r="52" spans="27:39" x14ac:dyDescent="0.35">
+    <row r="52" spans="27:56" x14ac:dyDescent="0.35">
       <c r="AA52" t="s">
         <v>0</v>
       </c>
       <c r="AI52" t="s">
         <v>82</v>
       </c>
+      <c r="AP52" s="10"/>
+      <c r="AQ52" s="10"/>
+      <c r="AR52" s="10"/>
+      <c r="AS52" s="10"/>
+      <c r="AT52" s="10"/>
+      <c r="AU52" s="10"/>
+      <c r="AV52" s="10"/>
+      <c r="AW52" s="10"/>
+      <c r="AX52" s="10"/>
+      <c r="AY52" s="10"/>
+      <c r="AZ52" s="10"/>
+      <c r="BA52" s="10"/>
+      <c r="BB52" s="10"/>
+      <c r="BC52" s="10"/>
+      <c r="BD52" s="10"/>
     </row>
-    <row r="53" spans="27:39" x14ac:dyDescent="0.35">
+    <row r="53" spans="27:56" x14ac:dyDescent="0.35">
       <c r="AA53" t="s">
         <v>1</v>
       </c>
+      <c r="AP53" s="10"/>
+      <c r="AQ53" s="10"/>
+      <c r="AR53" s="10"/>
+      <c r="AS53" s="10"/>
+      <c r="AT53" s="10"/>
+      <c r="AU53" s="10"/>
+      <c r="AV53" s="10"/>
+      <c r="AW53" s="10"/>
+      <c r="AX53" s="10"/>
+      <c r="AY53" s="10"/>
+      <c r="AZ53" s="10"/>
+      <c r="BA53" s="10"/>
+      <c r="BB53" s="10"/>
+      <c r="BC53" s="10"/>
+      <c r="BD53" s="10"/>
     </row>
-    <row r="54" spans="27:39" x14ac:dyDescent="0.35">
+    <row r="54" spans="27:56" x14ac:dyDescent="0.35">
       <c r="AA54" t="s">
         <v>2</v>
       </c>
+      <c r="AP54" s="10"/>
+      <c r="AQ54" s="10"/>
+      <c r="AR54" s="10"/>
+      <c r="AS54" s="10"/>
+      <c r="AT54" s="10"/>
+      <c r="AU54" s="10"/>
+      <c r="AV54" s="10"/>
+      <c r="AW54" s="10"/>
+      <c r="AX54" s="10"/>
+      <c r="AY54" s="10"/>
+      <c r="AZ54" s="10"/>
+      <c r="BA54" s="10"/>
+      <c r="BB54" s="10"/>
+      <c r="BC54" s="10"/>
+      <c r="BD54" s="10"/>
     </row>
-    <row r="55" spans="27:39" x14ac:dyDescent="0.35">
+    <row r="55" spans="27:56" x14ac:dyDescent="0.35">
       <c r="AA55" t="s">
         <v>3</v>
       </c>
+      <c r="AP55" s="10"/>
+      <c r="AQ55" s="10"/>
+      <c r="AR55" s="10"/>
+      <c r="AS55" s="10"/>
+      <c r="AT55" s="10"/>
+      <c r="AU55" s="10"/>
+      <c r="AV55" s="10"/>
+      <c r="AW55" s="10"/>
+      <c r="AX55" s="10"/>
+      <c r="AY55" s="10"/>
+      <c r="AZ55" s="10"/>
+      <c r="BA55" s="10"/>
+      <c r="BB55" s="10"/>
+      <c r="BC55" s="10"/>
+      <c r="BD55" s="10"/>
     </row>
-    <row r="56" spans="27:39" x14ac:dyDescent="0.35">
+    <row r="56" spans="27:56" x14ac:dyDescent="0.35">
       <c r="AA56" t="s">
         <v>4</v>
       </c>
       <c r="AI56" t="s">
         <v>83</v>
       </c>
+      <c r="AP56" s="10"/>
+      <c r="AQ56" s="10"/>
+      <c r="AR56" s="10"/>
+      <c r="AS56" s="10"/>
+      <c r="AT56" s="10"/>
+      <c r="AU56" s="10"/>
+      <c r="AV56" s="10"/>
+      <c r="AW56" s="10"/>
+      <c r="AX56" s="10"/>
+      <c r="AY56" s="10"/>
+      <c r="AZ56" s="10"/>
+      <c r="BA56" s="10"/>
+      <c r="BB56" s="10"/>
+      <c r="BC56" s="10"/>
+      <c r="BD56" s="10"/>
     </row>
-    <row r="57" spans="27:39" x14ac:dyDescent="0.35">
+    <row r="57" spans="27:56" x14ac:dyDescent="0.35">
       <c r="AI57" t="s">
         <v>84</v>
       </c>
+      <c r="AP57" s="10"/>
+      <c r="AQ57" s="10"/>
+      <c r="AR57" s="10"/>
+      <c r="AS57" s="10"/>
+      <c r="AT57" s="10"/>
+      <c r="AU57" s="10"/>
+      <c r="AV57" s="10"/>
+      <c r="AW57" s="10"/>
+      <c r="AX57" s="10"/>
+      <c r="AY57" s="10"/>
+      <c r="AZ57" s="10"/>
+      <c r="BA57" s="10"/>
+      <c r="BB57" s="10"/>
+      <c r="BC57" s="10"/>
+      <c r="BD57" s="10"/>
     </row>
-    <row r="58" spans="27:39" x14ac:dyDescent="0.35">
-      <c r="AA58" s="15" t="s">
+    <row r="58" spans="27:56" x14ac:dyDescent="0.35">
+      <c r="AA58" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="AB58" s="15"/>
-      <c r="AC58" s="15"/>
-      <c r="AD58" s="15"/>
-      <c r="AE58" s="15"/>
+      <c r="AB58" s="14"/>
+      <c r="AC58" s="14"/>
+      <c r="AD58" s="14"/>
+      <c r="AE58" s="14"/>
+      <c r="AP58" s="10"/>
+      <c r="AQ58" s="10"/>
+      <c r="AR58" s="10"/>
+      <c r="AS58" s="10"/>
+      <c r="AT58" s="10"/>
+      <c r="AU58" s="10"/>
+      <c r="AV58" s="10"/>
+      <c r="AW58" s="10"/>
+      <c r="AX58" s="10"/>
+      <c r="AY58" s="10"/>
+      <c r="AZ58" s="10"/>
+      <c r="BA58" s="10"/>
+      <c r="BB58" s="10"/>
+      <c r="BC58" s="10"/>
+      <c r="BD58" s="10"/>
     </row>
-    <row r="60" spans="27:39" x14ac:dyDescent="0.35">
+    <row r="59" spans="27:56" x14ac:dyDescent="0.35">
+      <c r="AP59" s="10"/>
+      <c r="AQ59" s="10"/>
+      <c r="AR59" s="10"/>
+      <c r="AS59" s="10"/>
+      <c r="AT59" s="10"/>
+      <c r="AU59" s="10"/>
+      <c r="AV59" s="10"/>
+      <c r="AW59" s="10"/>
+      <c r="AX59" s="10"/>
+      <c r="AY59" s="10"/>
+      <c r="AZ59" s="10"/>
+      <c r="BA59" s="10"/>
+      <c r="BB59" s="10"/>
+      <c r="BC59" s="10"/>
+      <c r="BD59" s="10"/>
+    </row>
+    <row r="60" spans="27:56" x14ac:dyDescent="0.35">
       <c r="AA60" t="s">
         <v>12</v>
       </c>
+      <c r="AP60" s="10"/>
+      <c r="AQ60" s="10"/>
+      <c r="AR60" s="10"/>
+      <c r="AS60" s="10"/>
+      <c r="AT60" s="10"/>
+      <c r="AU60" s="10"/>
+      <c r="AV60" s="10"/>
+      <c r="AW60" s="10"/>
+      <c r="AX60" s="10"/>
+      <c r="AY60" s="10"/>
+      <c r="AZ60" s="10"/>
+      <c r="BA60" s="10"/>
+      <c r="BB60" s="10"/>
+      <c r="BC60" s="10"/>
+      <c r="BD60" s="10"/>
     </row>
-    <row r="61" spans="27:39" x14ac:dyDescent="0.35">
+    <row r="61" spans="27:56" x14ac:dyDescent="0.35">
       <c r="AA61" t="s">
         <v>13</v>
       </c>
+      <c r="AP61" s="10"/>
+      <c r="AQ61" s="10"/>
+      <c r="AR61" s="10"/>
+      <c r="AS61" s="10"/>
+      <c r="AT61" s="10"/>
+      <c r="AU61" s="10"/>
+      <c r="AV61" s="10"/>
+      <c r="AW61" s="10"/>
+      <c r="AX61" s="10"/>
+      <c r="AY61" s="10"/>
+      <c r="AZ61" s="10"/>
+      <c r="BA61" s="10"/>
+      <c r="BB61" s="10"/>
+      <c r="BC61" s="10"/>
+      <c r="BD61" s="10"/>
     </row>
-    <row r="62" spans="27:39" x14ac:dyDescent="0.35">
+    <row r="62" spans="27:56" x14ac:dyDescent="0.35">
       <c r="AA62" t="s">
         <v>14</v>
       </c>
+      <c r="AP62" s="10"/>
+      <c r="AQ62" s="10"/>
+      <c r="AR62" s="10"/>
+      <c r="AS62" s="10"/>
+      <c r="AT62" s="10"/>
+      <c r="AU62" s="10"/>
+      <c r="AV62" s="10"/>
+      <c r="AW62" s="10"/>
+      <c r="AX62" s="10"/>
+      <c r="AY62" s="10"/>
+      <c r="AZ62" s="10"/>
+      <c r="BA62" s="10"/>
+      <c r="BB62" s="10"/>
+      <c r="BC62" s="10"/>
+      <c r="BD62" s="10"/>
     </row>
-    <row r="63" spans="27:39" x14ac:dyDescent="0.35">
+    <row r="63" spans="27:56" x14ac:dyDescent="0.35">
       <c r="AA63" t="s">
         <v>15</v>
       </c>
       <c r="AI63" t="s">
         <v>85</v>
       </c>
+      <c r="AP63" s="10"/>
+      <c r="AQ63" s="10"/>
+      <c r="AR63" s="10"/>
+      <c r="AS63" s="10"/>
+      <c r="AT63" s="10"/>
+      <c r="AU63" s="10"/>
+      <c r="AV63" s="10"/>
+      <c r="AW63" s="10"/>
+      <c r="AX63" s="10"/>
+      <c r="AY63" s="10"/>
+      <c r="AZ63" s="10"/>
+      <c r="BA63" s="10"/>
+      <c r="BB63" s="10"/>
+      <c r="BC63" s="10"/>
+      <c r="BD63" s="10"/>
     </row>
-    <row r="64" spans="27:39" x14ac:dyDescent="0.35">
+    <row r="64" spans="27:56" x14ac:dyDescent="0.35">
       <c r="AA64" t="s">
         <v>16</v>
       </c>
@@ -9407,6 +11288,21 @@
       <c r="AK64" s="9"/>
       <c r="AL64" s="9"/>
       <c r="AM64" s="9"/>
+      <c r="AP64" s="10"/>
+      <c r="AQ64" s="10"/>
+      <c r="AR64" s="10"/>
+      <c r="AS64" s="10"/>
+      <c r="AT64" s="10"/>
+      <c r="AU64" s="10"/>
+      <c r="AV64" s="10"/>
+      <c r="AW64" s="10"/>
+      <c r="AX64" s="10"/>
+      <c r="AY64" s="10"/>
+      <c r="AZ64" s="10"/>
+      <c r="BA64" s="10"/>
+      <c r="BB64" s="10"/>
+      <c r="BC64" s="10"/>
+      <c r="BD64" s="10"/>
     </row>
     <row r="65" spans="27:35" x14ac:dyDescent="0.35">
       <c r="AA65" t="s">
@@ -9450,7 +11346,8 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
+    <mergeCell ref="BG2:BL2"/>
     <mergeCell ref="B2:K2"/>
     <mergeCell ref="AQ2:BC2"/>
     <mergeCell ref="AA58:AE58"/>
@@ -9480,14 +11377,14 @@
   </cols>
   <sheetData>
     <row r="4" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="15"/>
-      <c r="D4" s="15"/>
-      <c r="E4" s="15"/>
-      <c r="F4" s="15"/>
-      <c r="G4" s="15"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
+      <c r="G4" s="14"/>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B6" t="s">

</xml_diff>